<commit_message>
DealLens phase 4: diligence intelligence
- rag/facts: normalised financial facts (concept/period/base-unit value) with page+cell provenance
- rag/diligence: contradiction finder (0.5%/rounding-aware, authority-ranked sides), table total checks,
  missing-reference detection, auto-drafted seller question list (ranked, grouped, cited)
- rag/packs: Financials / Contracts / Debt matrices (facts, typed tables, retrieval; no generation)
- rag/maturity: maturity wall with receipts + deal timeline (grouped, malformed dates ignored)
- rag/exports: CSV/XLSX/DOCX/Markdown with formula-injection protection
- API + UI: Contradictions, Packs, Seller Questions (editable, exportable), Maturity Wall
- demo data room gains a typed wrong total; tests: 17 new

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/project_falcon/Falcon_Management_Accounts.xlsx
+++ b/demo/project_falcon/Falcon_Management_Accounts.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t xml:space="preserve">Month</t>
   </si>
@@ -64,6 +64,9 @@
   </si>
   <si>
     <t xml:space="preserve">Mar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
   </si>
   <si>
     <t xml:space="preserve">Metric</t>
@@ -366,7 +369,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -471,6 +474,14 @@
       </c>
       <c r="B13" s="0" t="n">
         <v>40</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>449</v>
       </c>
     </row>
   </sheetData>
@@ -494,15 +505,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B2" s="0" t="n">
         <f aca="false">SUM(Monthly!B2:B13)</f>
@@ -511,7 +522,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B3" s="0" t="n">
         <v>383</v>
@@ -519,7 +530,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" s="0" t="n">
         <f aca="false">B2-B3</f>
@@ -528,7 +539,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B5" s="0" t="n">
         <v>84</v>
@@ -536,7 +547,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B6" s="0" t="n">
         <v>48.2</v>
@@ -563,15 +574,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B2" s="0" t="n">
         <v>15</v>

</xml_diff>